<commit_message>
Mise à jour de l'application
</commit_message>
<xml_diff>
--- a/data/2026-2027/DonneesGPSPropres.xlsx
+++ b/data/2026-2027/DonneesGPSPropres.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christophergallo/Desktop/Application perso/data/2026-2027/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D240773-116B-8649-8C41-AC7006DE6528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DF093EE-B65D-4746-9E9C-88146D034048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16360" xr2:uid="{D839DFFF-AA38-2145-9D48-3C82EEA1EE91}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="56">
   <si>
     <t>Temps joué</t>
   </si>
@@ -130,9 +130,6 @@
     <t>Karahali Souaré</t>
   </si>
   <si>
-    <t>Yoan Zouma</t>
-  </si>
-  <si>
     <t>Mattheo Haon</t>
   </si>
   <si>
@@ -176,13 +173,43 @@
   </si>
   <si>
     <t>01:08:52</t>
+  </si>
+  <si>
+    <t>Ryad Kralladi</t>
+  </si>
+  <si>
+    <t>01:10:58</t>
+  </si>
+  <si>
+    <t>01:10:25</t>
+  </si>
+  <si>
+    <t>01:11:52</t>
+  </si>
+  <si>
+    <t>01:08:58</t>
+  </si>
+  <si>
+    <t>01:11:39</t>
+  </si>
+  <si>
+    <t>01:09:18</t>
+  </si>
+  <si>
+    <t>Gibril Djahl</t>
+  </si>
+  <si>
+    <t>01:08:04</t>
+  </si>
+  <si>
+    <t>01:12:07</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -195,6 +222,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -217,7 +250,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -226,6 +259,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -540,7 +574,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3AE8228-0F81-ED4B-A4A4-4C340123FE2A}">
-  <dimension ref="A1:V10"/>
+  <dimension ref="A1:V19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" customWidth="1"/>
@@ -628,13 +662,13 @@
         <v>19</v>
       </c>
       <c r="E2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
         <v>27</v>
       </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H2">
         <v>7</v>
@@ -693,13 +727,13 @@
         <v>19</v>
       </c>
       <c r="E3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F3" t="s">
         <v>26</v>
       </c>
       <c r="G3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H3">
         <v>7.41</v>
@@ -758,13 +792,13 @@
         <v>19</v>
       </c>
       <c r="E4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F4" t="s">
         <v>28</v>
       </c>
       <c r="G4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H4">
         <v>6.91</v>
@@ -829,7 +863,7 @@
         <v>26</v>
       </c>
       <c r="G5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H5">
         <v>6.88</v>
@@ -888,13 +922,13 @@
         <v>19</v>
       </c>
       <c r="E6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F6" t="s">
         <v>27</v>
       </c>
       <c r="G6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H6">
         <v>7.31</v>
@@ -953,13 +987,13 @@
         <v>19</v>
       </c>
       <c r="E7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F7" t="s">
         <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H7">
         <v>7.38</v>
@@ -1018,13 +1052,13 @@
         <v>19</v>
       </c>
       <c r="E8" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="F8" t="s">
         <v>24</v>
       </c>
       <c r="G8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H8">
         <v>7.01</v>
@@ -1083,13 +1117,13 @@
         <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F9" t="s">
         <v>27</v>
       </c>
       <c r="G9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H9">
         <v>6.84</v>
@@ -1154,7 +1188,7 @@
         <v>25</v>
       </c>
       <c r="G10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H10">
         <v>6.45</v>
@@ -1199,6 +1233,591 @@
         <v>3</v>
       </c>
       <c r="V10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="1">
+        <v>46217</v>
+      </c>
+      <c r="C11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" t="s">
+        <v>47</v>
+      </c>
+      <c r="H11">
+        <v>6.27</v>
+      </c>
+      <c r="I11">
+        <v>0.73</v>
+      </c>
+      <c r="J11">
+        <v>5.53</v>
+      </c>
+      <c r="K11">
+        <v>0.74</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <v>5.29</v>
+      </c>
+      <c r="Q11">
+        <v>18.64</v>
+      </c>
+      <c r="R11">
+        <v>3.44</v>
+      </c>
+      <c r="S11">
+        <v>5</v>
+      </c>
+      <c r="T11">
+        <v>0</v>
+      </c>
+      <c r="U11">
+        <v>5</v>
+      </c>
+      <c r="V11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="1">
+        <v>46217</v>
+      </c>
+      <c r="C12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" t="s">
+        <v>48</v>
+      </c>
+      <c r="H12">
+        <v>7.06</v>
+      </c>
+      <c r="I12">
+        <v>0.84</v>
+      </c>
+      <c r="J12">
+        <v>6.21</v>
+      </c>
+      <c r="K12">
+        <v>0.84</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12">
+        <v>0</v>
+      </c>
+      <c r="P12">
+        <v>5.96</v>
+      </c>
+      <c r="Q12">
+        <v>19.91</v>
+      </c>
+      <c r="R12">
+        <v>4.25</v>
+      </c>
+      <c r="S12">
+        <v>11</v>
+      </c>
+      <c r="T12">
+        <v>1</v>
+      </c>
+      <c r="U12">
+        <v>1</v>
+      </c>
+      <c r="V12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="1">
+        <v>46217</v>
+      </c>
+      <c r="C13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" t="s">
+        <v>49</v>
+      </c>
+      <c r="H13">
+        <v>7.07</v>
+      </c>
+      <c r="I13">
+        <v>1.24</v>
+      </c>
+      <c r="J13">
+        <v>5.83</v>
+      </c>
+      <c r="K13">
+        <v>1.23</v>
+      </c>
+      <c r="L13">
+        <v>0.01</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13">
+        <v>1</v>
+      </c>
+      <c r="P13">
+        <v>5.86</v>
+      </c>
+      <c r="Q13">
+        <v>25.12</v>
+      </c>
+      <c r="R13">
+        <v>4.47</v>
+      </c>
+      <c r="S13">
+        <v>10</v>
+      </c>
+      <c r="T13">
+        <v>3</v>
+      </c>
+      <c r="U13">
+        <v>4</v>
+      </c>
+      <c r="V13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="1">
+        <v>46217</v>
+      </c>
+      <c r="C14" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" t="s">
+        <v>25</v>
+      </c>
+      <c r="G14" t="s">
+        <v>50</v>
+      </c>
+      <c r="H14">
+        <v>6.53</v>
+      </c>
+      <c r="I14">
+        <v>0.47</v>
+      </c>
+      <c r="J14">
+        <v>6.05</v>
+      </c>
+      <c r="K14">
+        <v>0.49</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="P14">
+        <v>5.2</v>
+      </c>
+      <c r="Q14">
+        <v>18.399999999999999</v>
+      </c>
+      <c r="R14">
+        <v>4.59</v>
+      </c>
+      <c r="S14">
+        <v>15</v>
+      </c>
+      <c r="T14">
+        <v>2</v>
+      </c>
+      <c r="U14">
+        <v>7</v>
+      </c>
+      <c r="V14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="1">
+        <v>46217</v>
+      </c>
+      <c r="C15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F15" t="s">
+        <v>28</v>
+      </c>
+      <c r="G15" t="s">
+        <v>50</v>
+      </c>
+      <c r="H15">
+        <v>6.69</v>
+      </c>
+      <c r="I15">
+        <v>0.63</v>
+      </c>
+      <c r="J15">
+        <v>6.06</v>
+      </c>
+      <c r="K15">
+        <v>0.63</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15">
+        <v>5.81</v>
+      </c>
+      <c r="Q15">
+        <v>18.510000000000002</v>
+      </c>
+      <c r="R15">
+        <v>4.22</v>
+      </c>
+      <c r="S15">
+        <v>17</v>
+      </c>
+      <c r="T15">
+        <v>2</v>
+      </c>
+      <c r="U15">
+        <v>8</v>
+      </c>
+      <c r="V15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="1">
+        <v>46217</v>
+      </c>
+      <c r="C16" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" t="s">
+        <v>43</v>
+      </c>
+      <c r="F16" t="s">
+        <v>24</v>
+      </c>
+      <c r="G16" t="s">
+        <v>51</v>
+      </c>
+      <c r="H16">
+        <v>7.56</v>
+      </c>
+      <c r="I16">
+        <v>1.66</v>
+      </c>
+      <c r="J16">
+        <v>5.9</v>
+      </c>
+      <c r="K16">
+        <v>1.64</v>
+      </c>
+      <c r="L16">
+        <v>0.02</v>
+      </c>
+      <c r="M16">
+        <v>0</v>
+      </c>
+      <c r="N16">
+        <v>0</v>
+      </c>
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16">
+        <v>6.28</v>
+      </c>
+      <c r="Q16">
+        <v>22.7</v>
+      </c>
+      <c r="R16">
+        <v>4.3899999999999997</v>
+      </c>
+      <c r="S16">
+        <v>22</v>
+      </c>
+      <c r="T16">
+        <v>4</v>
+      </c>
+      <c r="U16">
+        <v>1</v>
+      </c>
+      <c r="V16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="1">
+        <v>46217</v>
+      </c>
+      <c r="C17" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" t="s">
+        <v>35</v>
+      </c>
+      <c r="F17" t="s">
+        <v>27</v>
+      </c>
+      <c r="G17" t="s">
+        <v>52</v>
+      </c>
+      <c r="H17">
+        <v>6.58</v>
+      </c>
+      <c r="I17">
+        <v>0.79</v>
+      </c>
+      <c r="J17">
+        <v>5.79</v>
+      </c>
+      <c r="K17">
+        <v>0.79</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17">
+        <v>0</v>
+      </c>
+      <c r="N17">
+        <v>0</v>
+      </c>
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="P17">
+        <v>5.66</v>
+      </c>
+      <c r="Q17">
+        <v>19.21</v>
+      </c>
+      <c r="R17">
+        <v>3.82</v>
+      </c>
+      <c r="S17">
+        <v>14</v>
+      </c>
+      <c r="T17">
+        <v>0</v>
+      </c>
+      <c r="U17">
+        <v>1</v>
+      </c>
+      <c r="V17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="1">
+        <v>46217</v>
+      </c>
+      <c r="C18" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" t="s">
+        <v>53</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G18" t="s">
+        <v>54</v>
+      </c>
+      <c r="H18">
+        <v>5.26</v>
+      </c>
+      <c r="I18">
+        <v>0.05</v>
+      </c>
+      <c r="J18">
+        <v>5.21</v>
+      </c>
+      <c r="K18">
+        <v>0.05</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>0</v>
+      </c>
+      <c r="N18">
+        <v>0</v>
+      </c>
+      <c r="O18">
+        <v>0</v>
+      </c>
+      <c r="P18">
+        <v>4.68</v>
+      </c>
+      <c r="Q18">
+        <v>16.579999999999998</v>
+      </c>
+      <c r="R18">
+        <v>3.25</v>
+      </c>
+      <c r="S18">
+        <v>5</v>
+      </c>
+      <c r="T18">
+        <v>0</v>
+      </c>
+      <c r="U18">
+        <v>2</v>
+      </c>
+      <c r="V18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="1">
+        <v>46217</v>
+      </c>
+      <c r="C19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" t="s">
+        <v>36</v>
+      </c>
+      <c r="F19" t="s">
+        <v>26</v>
+      </c>
+      <c r="G19" t="s">
+        <v>55</v>
+      </c>
+      <c r="H19">
+        <v>6.96</v>
+      </c>
+      <c r="I19">
+        <v>1.18</v>
+      </c>
+      <c r="J19">
+        <v>5.78</v>
+      </c>
+      <c r="K19">
+        <v>1.17</v>
+      </c>
+      <c r="L19">
+        <v>0.01</v>
+      </c>
+      <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="N19">
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <v>5.73</v>
+      </c>
+      <c r="Q19">
+        <v>20.28</v>
+      </c>
+      <c r="R19">
+        <v>3.73</v>
+      </c>
+      <c r="S19">
+        <v>5</v>
+      </c>
+      <c r="T19">
+        <v>0</v>
+      </c>
+      <c r="U19">
+        <v>3</v>
+      </c>
+      <c r="V19">
         <v>0</v>
       </c>
     </row>

</xml_diff>